<commit_message>
re-render F04/F05 on the raw F03 cache so concordance reads the full symmetric NES set
</commit_message>
<xml_diff>
--- a/04_Figures/extras/concordance_acute/c_data/F05_source_data.xlsx
+++ b/04_Figures/extras/concordance_acute/c_data/F05_source_data.xlsx
@@ -6121,163 +6121,163 @@
     <t xml:space="preserve">class</t>
   </si>
   <si>
+    <t xml:space="preserve">GOSLIM_AMINO_ACID_METABOLIC_PROCESS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GO Slim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concordant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_CHROMOSOME_SEGREGATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_CILIUM_ORGANIZATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_CYTOKINESIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_CYTOPLASMIC_TRANSLATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_DETOXIFICATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_DNA_RECOMBINATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_DNA_REPLICATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_ESTABLISHMENT_OR_MAINTENANCE_OF_CELL_POLARITY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_EXTRACELLULAR_MATRIX_ORGANIZATION</t>
+  </si>
+  <si>
     <t xml:space="preserve">GOSLIM_GENERATION_OF_PRECURSOR_METABOLITES_AND_ENERGY</t>
   </si>
   <si>
-    <t xml:space="preserve">GO Slim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_CYTOPLASMIC_TRANSLATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concordant</t>
+    <t xml:space="preserve">GOSLIM_GLYCOPROTEIN_METABOLIC_PROCESS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_KETONE_METABOLIC_PROCESS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_MICROTUBULE-BASED_MOVEMENT</t>
   </si>
   <si>
     <t xml:space="preserve">GOSLIM_MITOCHONDRION_ORGANIZATION</t>
   </si>
   <si>
+    <t xml:space="preserve">GOSLIM_MITOTIC_NUCLEAR_DIVISION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_MUSCLE_SYSTEM_PROCESS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_NUCLEOCYTOPLASMIC_TRANSPORT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_PROTEIN_FOLDING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_RIBOSOME_BIOGENESIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_TELOMERE_ORGANIZATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_TRNA_METABOLIC_PROCESS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOSLIM_WOUND_HEALING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_ADIPOGENESIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_ALLOGRAFT_REJECTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_ANDROGEN_RESPONSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_APICAL_JUNCTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_APOPTOSIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_BILE_ACID_METABOLISM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_COAGULATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_COMPLEMENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_DNA_REPAIR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_E2F_TARGETS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_EPITHELIAL_MESENCHYMAL_TRANSITION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_ESTROGEN_RESPONSE_EARLY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_ESTROGEN_RESPONSE_LATE</t>
+  </si>
+  <si>
     <t xml:space="preserve">HALLMARK_G2M_CHECKPOINT</t>
   </si>
   <si>
-    <t xml:space="preserve">HALLMARK_ADIPOGENESIS</t>
+    <t xml:space="preserve">HALLMARK_GLYCOLYSIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_HYPOXIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_IL2_STAT5_SIGNALING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_INTERFERON_GAMMA_RESPONSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_MITOTIC_SPINDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_MTORC1_SIGNALING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_MYOGENESIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_P53_PATHWAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_PEROXISOME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_PI3K_AKT_MTOR_SIGNALING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_PROTEIN_SECRETION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_REACTIVE_OXYGEN_SPECIES_PATHWAY</t>
   </si>
   <si>
     <t xml:space="preserve">HALLMARK_UNFOLDED_PROTEIN_RESPONSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_AMINO_ACID_METABOLIC_PROCESS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_MUSCLE_SYSTEM_PROCESS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_MITOTIC_SPINDLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_ESTABLISHMENT_OR_MAINTENANCE_OF_CELL_POLARITY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_E2F_TARGETS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_GLYCOLYSIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_TELOMERE_ORGANIZATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_RIBOSOME_BIOGENESIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_DNA_REPLICATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_NUCLEOCYTOPLASMIC_TRANSPORT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_CHROMOSOME_SEGREGATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_CILIUM_ORGANIZATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_CYTOKINESIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_DETOXIFICATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_DNA_RECOMBINATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_EXTRACELLULAR_MATRIX_ORGANIZATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_GLYCOPROTEIN_METABOLIC_PROCESS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_KETONE_METABOLIC_PROCESS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_MICROTUBULE-BASED_MOVEMENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_MITOTIC_NUCLEAR_DIVISION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_PROTEIN_FOLDING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_TRNA_METABOLIC_PROCESS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOSLIM_WOUND_HEALING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_ALLOGRAFT_REJECTION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_ANDROGEN_RESPONSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_APICAL_JUNCTION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_APOPTOSIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_BILE_ACID_METABOLISM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_COAGULATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_COMPLEMENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_DNA_REPAIR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_EPITHELIAL_MESENCHYMAL_TRANSITION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_ESTROGEN_RESPONSE_EARLY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_ESTROGEN_RESPONSE_LATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_HYPOXIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_IL2_STAT5_SIGNALING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_INTERFERON_GAMMA_RESPONSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_MTORC1_SIGNALING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_MYOGENESIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_P53_PATHWAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_PEROXISOME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_PI3K_AKT_MTOR_SIGNALING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_PROTEIN_SECRETION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HALLMARK_REACTIVE_OXYGEN_SPECIES_PATHWAY</t>
   </si>
   <si>
     <t xml:space="preserve">HALLMARK_UV_RESPONSE_UP</t>
@@ -60154,137 +60154,137 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1939</v>
+        <v>2033</v>
       </c>
       <c r="B2" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C2" t="n">
-        <v>-2.65625893338279</v>
+        <v>-1.809725642848</v>
       </c>
       <c r="D2" t="n">
-        <v>-1.38159490915102</v>
+        <v>-0.742894405628763</v>
       </c>
       <c r="E2" t="n">
-        <v>0.000000000000947150908861262</v>
+        <v>0.00260145072530896</v>
       </c>
       <c r="F2" t="n">
-        <v>0.207765658228716</v>
+        <v>0.984184015181113</v>
       </c>
       <c r="G2" t="n">
-        <v>152</v>
+        <v>95</v>
       </c>
       <c r="H2" t="n">
-        <v>152</v>
+        <v>95</v>
       </c>
       <c r="I2" t="n">
-        <v>152</v>
+        <v>95</v>
       </c>
       <c r="J2" t="n">
-        <v>-1.79082687996285</v>
+        <v>-1.51788931199482</v>
       </c>
       <c r="K2" t="n">
-        <v>0.00189151757306219</v>
+        <v>0.0858861316634714</v>
       </c>
       <c r="L2" t="n">
-        <v>-2.65625893338279</v>
+        <v>-1.809725642848</v>
       </c>
       <c r="M2" t="n">
-        <v>-1.38159490915102</v>
+        <v>-0.742894405628763</v>
       </c>
       <c r="N2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>33</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2033</v>
+        <v>2036</v>
       </c>
       <c r="B3" t="s">
         <v>2034</v>
       </c>
       <c r="C3" t="n">
-        <v>-2.45244421962224</v>
+        <v>1.35582515562311</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.31638809317296</v>
+        <v>-0.882405625012737</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0000000000120358134557067</v>
+        <v>0.211816468982289</v>
       </c>
       <c r="F3" t="n">
-        <v>0.220531267293857</v>
+        <v>0.921121127858664</v>
       </c>
       <c r="G3" t="n">
-        <v>210</v>
+        <v>52</v>
       </c>
       <c r="H3" t="n">
-        <v>210</v>
+        <v>51</v>
       </c>
       <c r="I3" t="n">
-        <v>210</v>
+        <v>52</v>
       </c>
       <c r="J3" t="n">
-        <v>-1.78491614885634</v>
+        <v>1.44666817087964</v>
       </c>
       <c r="K3" t="n">
-        <v>0.000960249468853041</v>
+        <v>0.209468580200288</v>
       </c>
       <c r="L3" t="n">
-        <v>-2.45244421962224</v>
+        <v>1.35582515562311</v>
       </c>
       <c r="M3" t="n">
-        <v>-1.31638809317296</v>
+        <v>-0.882405625012737</v>
       </c>
       <c r="N3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>33</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2035</v>
+        <v>2037</v>
       </c>
       <c r="B4" t="s">
         <v>2034</v>
       </c>
       <c r="C4" t="n">
-        <v>2.39769229466252</v>
+        <v>1.65381155921971</v>
       </c>
       <c r="D4" t="n">
-        <v>1.03386572985999</v>
+        <v>-1.41637962553889</v>
       </c>
       <c r="E4" t="n">
-        <v>0.000000050756419272981</v>
+        <v>0.0598891942337842</v>
       </c>
       <c r="F4" t="n">
-        <v>0.780326534897761</v>
+        <v>0.4479677747983</v>
       </c>
       <c r="G4" t="n">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="H4" t="n">
-        <v>114</v>
+        <v>31</v>
       </c>
       <c r="I4" t="n">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="J4" t="n">
-        <v>1.97657075593812</v>
+        <v>1.88161559233992</v>
       </c>
       <c r="K4" t="n">
-        <v>0.000678601852834159</v>
+        <v>0.0174534983302519</v>
       </c>
       <c r="L4" t="n">
-        <v>2.39769229466252</v>
+        <v>1.65381155921971</v>
       </c>
       <c r="M4" t="n">
-        <v>1.03386572985999</v>
+        <v>-1.41637962553889</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -60295,1970 +60295,1970 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1928</v>
+        <v>2038</v>
       </c>
       <c r="B5" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C5" t="n">
-        <v>2.17641704034345</v>
+        <v>0.778887100366341</v>
       </c>
       <c r="D5" t="n">
-        <v>1.72909466449593</v>
+        <v>-1.02035245356723</v>
       </c>
       <c r="E5" t="n">
-        <v>0.00000430594823680413</v>
+        <v>0.946882388254389</v>
       </c>
       <c r="F5" t="n">
-        <v>0.024475642139805</v>
+        <v>0.790937182749941</v>
       </c>
       <c r="G5" t="n">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="H5" t="n">
-        <v>118</v>
+        <v>37</v>
       </c>
       <c r="I5" t="n">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="J5" t="n">
-        <v>1.31472586306208</v>
+        <v>1.14808621787384</v>
       </c>
       <c r="K5" t="n">
-        <v>0.253696621162633</v>
+        <v>0.534198335931694</v>
       </c>
       <c r="L5" t="n">
-        <v>2.17641704034345</v>
+        <v>0.778887100366341</v>
       </c>
       <c r="M5" t="n">
-        <v>1.72909466449593</v>
+        <v>-1.02035245356723</v>
       </c>
       <c r="N5" t="b">
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="B6" t="s">
         <v>2034</v>
       </c>
       <c r="C6" t="n">
-        <v>-2.09470201300686</v>
+        <v>2.39769229466252</v>
       </c>
       <c r="D6" t="n">
-        <v>-1.36068950182374</v>
+        <v>1.03386572985999</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0000103885408014993</v>
+        <v>0.000000050756419272981</v>
       </c>
       <c r="F6" t="n">
-        <v>0.273585445391613</v>
+        <v>0.780326534897761</v>
       </c>
       <c r="G6" t="n">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="H6" t="n">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I6" t="n">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.41725327451678</v>
+        <v>1.97657075593812</v>
       </c>
       <c r="K6" t="n">
-        <v>0.138394668212112</v>
+        <v>0.000678601852834159</v>
       </c>
       <c r="L6" t="n">
-        <v>-2.09470201300686</v>
+        <v>2.39769229466252</v>
       </c>
       <c r="M6" t="n">
-        <v>-1.36068950182374</v>
+        <v>1.03386572985999</v>
       </c>
       <c r="N6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" t="s">
-        <v>2036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1949</v>
+        <v>2040</v>
       </c>
       <c r="B7" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.09530870215646</v>
+        <v>-1.01520257747063</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.88328325844714</v>
+        <v>1.19424185389282</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0000737780828421685</v>
+        <v>0.676421561638628</v>
       </c>
       <c r="F7" t="n">
-        <v>0.924770700656501</v>
+        <v>0.626700486918879</v>
       </c>
       <c r="G7" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="H7" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="J7" t="n">
-        <v>-1.71677175976851</v>
+        <v>-1.2156753146664</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0174534983302519</v>
+        <v>0.441817448772222</v>
       </c>
       <c r="L7" t="n">
-        <v>-2.09530870215646</v>
+        <v>-1.01520257747063</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.88328325844714</v>
+        <v>1.19424185389282</v>
       </c>
       <c r="N7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>33</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2038</v>
+        <v>2041</v>
       </c>
       <c r="B8" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C8" t="n">
-        <v>2.19134060699225</v>
+        <v>1.44828403462988</v>
       </c>
       <c r="D8" t="n">
-        <v>1.0754110538426</v>
+        <v>1.32822540349866</v>
       </c>
       <c r="E8" t="n">
-        <v>0.000645051063205934</v>
+        <v>0.188568291897933</v>
       </c>
       <c r="F8" t="n">
-        <v>0.746714126712962</v>
+        <v>0.544583416703077</v>
       </c>
       <c r="G8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J8" t="n">
-        <v>1.95896018601054</v>
+        <v>-0.971477774753253</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0145465812893292</v>
+        <v>0.719625587265655</v>
       </c>
       <c r="L8" t="n">
-        <v>2.19134060699225</v>
+        <v>1.44828403462988</v>
       </c>
       <c r="M8" t="n">
-        <v>1.0754110538426</v>
+        <v>1.32822540349866</v>
       </c>
       <c r="N8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" t="s">
-        <v>33</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2039</v>
+        <v>2042</v>
       </c>
       <c r="B9" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C9" t="n">
-        <v>-1.86946782709568</v>
+        <v>1.73927995059662</v>
       </c>
       <c r="D9" t="n">
-        <v>0.719963677893052</v>
+        <v>-0.813098905337296</v>
       </c>
       <c r="E9" t="n">
-        <v>0.00203304443414014</v>
+        <v>0.0417432010170257</v>
       </c>
       <c r="F9" t="n">
-        <v>0.983333938876475</v>
+        <v>0.93386330867079</v>
       </c>
       <c r="G9" t="n">
-        <v>96</v>
+        <v>31</v>
       </c>
       <c r="H9" t="n">
-        <v>96</v>
+        <v>31</v>
       </c>
       <c r="I9" t="n">
-        <v>96</v>
+        <v>31</v>
       </c>
       <c r="J9" t="n">
-        <v>-1.657593732751</v>
+        <v>1.44422832824758</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0172251263037516</v>
+        <v>0.236574279605685</v>
       </c>
       <c r="L9" t="n">
-        <v>-1.86946782709568</v>
+        <v>1.73927995059662</v>
       </c>
       <c r="M9" t="n">
-        <v>0.719963677893052</v>
+        <v>-0.813098905337296</v>
       </c>
       <c r="N9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>33</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2040</v>
+        <v>2043</v>
       </c>
       <c r="B10" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C10" t="n">
-        <v>2.0843779279202</v>
+        <v>1.87526150525616</v>
       </c>
       <c r="D10" t="n">
-        <v>-1.13354216006671</v>
+        <v>1.35525461267368</v>
       </c>
       <c r="E10" t="n">
-        <v>0.00214014985753382</v>
+        <v>0.00760432218828131</v>
       </c>
       <c r="F10" t="n">
-        <v>0.691622761470133</v>
+        <v>0.504716195047162</v>
       </c>
       <c r="G10" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H10" t="n">
         <v>34</v>
       </c>
       <c r="I10" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J10" t="n">
-        <v>2.17554919441156</v>
+        <v>1.23202665534272</v>
       </c>
       <c r="K10" t="n">
-        <v>0.00157336216247884</v>
+        <v>0.445122120647976</v>
       </c>
       <c r="L10" t="n">
-        <v>2.0843779279202</v>
+        <v>1.87526150525616</v>
       </c>
       <c r="M10" t="n">
-        <v>-1.13354216006671</v>
+        <v>1.35525461267368</v>
       </c>
       <c r="N10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O10" t="s">
-        <v>33</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2041</v>
+        <v>2044</v>
       </c>
       <c r="B11" t="s">
         <v>2034</v>
       </c>
       <c r="C11" t="n">
-        <v>-1.809725642848</v>
+        <v>-0.952503237797728</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.742894405628763</v>
+        <v>0.687548992153339</v>
       </c>
       <c r="E11" t="n">
-        <v>0.00260145072530896</v>
+        <v>0.761647518500162</v>
       </c>
       <c r="F11" t="n">
-        <v>0.984184015181113</v>
+        <v>0.96110820624015</v>
       </c>
       <c r="G11" t="n">
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="H11" t="n">
-        <v>95</v>
+        <v>19</v>
       </c>
       <c r="I11" t="n">
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="J11" t="n">
-        <v>-1.51788931199482</v>
+        <v>0.659655088775691</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0858861316634714</v>
+        <v>0.965520270340095</v>
       </c>
       <c r="L11" t="n">
-        <v>-1.809725642848</v>
+        <v>-0.952503237797728</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.742894405628763</v>
+        <v>0.687548992153339</v>
       </c>
       <c r="N11" t="b">
         <v>0</v>
       </c>
       <c r="O11" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2042</v>
+        <v>2045</v>
       </c>
       <c r="B12" t="s">
         <v>2034</v>
       </c>
       <c r="C12" t="n">
-        <v>1.70533676638263</v>
+        <v>-2.45244421962224</v>
       </c>
       <c r="D12" t="n">
-        <v>0.816529733149712</v>
+        <v>-1.31638809317296</v>
       </c>
       <c r="E12" t="n">
-        <v>0.00442569607457395</v>
+        <v>0.0000000000120358134557067</v>
       </c>
       <c r="F12" t="n">
-        <v>0.960149675132128</v>
+        <v>0.220531267293857</v>
       </c>
       <c r="G12" t="n">
-        <v>160</v>
+        <v>210</v>
       </c>
       <c r="H12" t="n">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="I12" t="n">
-        <v>160</v>
+        <v>210</v>
       </c>
       <c r="J12" t="n">
-        <v>1.493749171112</v>
+        <v>-1.78491614885634</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0730069508591943</v>
+        <v>0.000960249468853041</v>
       </c>
       <c r="L12" t="n">
-        <v>1.70533676638263</v>
+        <v>-2.45244421962224</v>
       </c>
       <c r="M12" t="n">
-        <v>0.816529733149712</v>
+        <v>-1.31638809317296</v>
       </c>
       <c r="N12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" t="s">
-        <v>2036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2043</v>
+        <v>2046</v>
       </c>
       <c r="B13" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C13" t="n">
-        <v>1.97676024961818</v>
+        <v>1.02438520348949</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.653603238796788</v>
+        <v>1.269710113962</v>
       </c>
       <c r="E13" t="n">
-        <v>0.00482063296372364</v>
+        <v>0.661729418167425</v>
       </c>
       <c r="F13" t="n">
-        <v>0.983333938876475</v>
+        <v>0.600030808751421</v>
       </c>
       <c r="G13" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="H13" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="I13" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="J13" t="n">
-        <v>1.83429777592081</v>
+        <v>0.927750307494303</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0272926051995232</v>
+        <v>0.767497746224927</v>
       </c>
       <c r="L13" t="n">
-        <v>1.97676024961818</v>
+        <v>1.02438520348949</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.653603238796788</v>
+        <v>1.269710113962</v>
       </c>
       <c r="N13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O13" t="s">
-        <v>33</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2044</v>
+        <v>2047</v>
       </c>
       <c r="B14" t="s">
         <v>2034</v>
       </c>
       <c r="C14" t="n">
-        <v>1.87526150525616</v>
+        <v>-1.26575924723775</v>
       </c>
       <c r="D14" t="n">
-        <v>1.35525461267368</v>
+        <v>-1.11282892008527</v>
       </c>
       <c r="E14" t="n">
-        <v>0.00760432218828131</v>
+        <v>0.305264847801037</v>
       </c>
       <c r="F14" t="n">
-        <v>0.504716195047162</v>
+        <v>0.70004508641563</v>
       </c>
       <c r="G14" t="n">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="H14" t="n">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="I14" t="n">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="J14" t="n">
-        <v>1.23202665534272</v>
+        <v>-0.704426086591038</v>
       </c>
       <c r="K14" t="n">
-        <v>0.445122120647976</v>
+        <v>0.969625345538602</v>
       </c>
       <c r="L14" t="n">
-        <v>1.87526150525616</v>
+        <v>-1.26575924723775</v>
       </c>
       <c r="M14" t="n">
-        <v>1.35525461267368</v>
+        <v>-1.11282892008527</v>
       </c>
       <c r="N14" t="b">
         <v>0</v>
       </c>
       <c r="O14" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2045</v>
+        <v>2048</v>
       </c>
       <c r="B15" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C15" t="n">
-        <v>1.8999377038983</v>
+        <v>1.08224870181928</v>
       </c>
       <c r="D15" t="n">
-        <v>1.87146635592682</v>
+        <v>1.09639280233169</v>
       </c>
       <c r="E15" t="n">
-        <v>0.00888284792363617</v>
+        <v>0.56628562092442</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0446591031563833</v>
+        <v>0.733451075800617</v>
       </c>
       <c r="G15" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="H15" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="I15" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="J15" t="n">
-        <v>1.04770669503782</v>
+        <v>-0.839141635339801</v>
       </c>
       <c r="K15" t="n">
-        <v>0.641277702659038</v>
+        <v>0.901552379611377</v>
       </c>
       <c r="L15" t="n">
-        <v>1.8999377038983</v>
+        <v>1.08224870181928</v>
       </c>
       <c r="M15" t="n">
-        <v>1.87146635592682</v>
+        <v>1.09639280233169</v>
       </c>
       <c r="N15" t="b">
         <v>0</v>
       </c>
       <c r="O15" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2046</v>
+        <v>2049</v>
       </c>
       <c r="B16" t="s">
-        <v>1930</v>
+        <v>2034</v>
       </c>
       <c r="C16" t="n">
-        <v>-1.76363136225828</v>
+        <v>-2.09470201300686</v>
       </c>
       <c r="D16" t="n">
-        <v>0.873534564896149</v>
+        <v>-1.36068950182374</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0114942849232801</v>
+        <v>0.0000103885408014993</v>
       </c>
       <c r="F16" t="n">
-        <v>0.921121127858664</v>
+        <v>0.273585445391613</v>
       </c>
       <c r="G16" t="n">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="H16" t="n">
-        <v>59</v>
+        <v>121</v>
       </c>
       <c r="I16" t="n">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="J16" t="n">
-        <v>-1.64855500834541</v>
+        <v>-1.41725327451678</v>
       </c>
       <c r="K16" t="n">
-        <v>0.0736698325163399</v>
+        <v>0.138394668212112</v>
       </c>
       <c r="L16" t="n">
-        <v>-1.76363136225828</v>
+        <v>-2.09470201300686</v>
       </c>
       <c r="M16" t="n">
-        <v>0.873534564896149</v>
+        <v>-1.36068950182374</v>
       </c>
       <c r="N16" t="b">
         <v>0</v>
       </c>
       <c r="O16" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2047</v>
+        <v>2050</v>
       </c>
       <c r="B17" t="s">
         <v>2034</v>
       </c>
       <c r="C17" t="n">
-        <v>1.81303144165592</v>
+        <v>1.01688459917931</v>
       </c>
       <c r="D17" t="n">
-        <v>1.93763983498075</v>
+        <v>-0.70477020001314</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0275455771583975</v>
+        <v>0.683226247706747</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0180933176598545</v>
+        <v>0.97728842555668</v>
       </c>
       <c r="G17" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="H17" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="I17" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.764179060682097</v>
+        <v>1.19954274745593</v>
       </c>
       <c r="K17" t="n">
-        <v>0.949223297337906</v>
+        <v>0.478461848697783</v>
       </c>
       <c r="L17" t="n">
-        <v>1.81303144165592</v>
+        <v>1.01688459917931</v>
       </c>
       <c r="M17" t="n">
-        <v>1.93763983498075</v>
+        <v>-0.70477020001314</v>
       </c>
       <c r="N17" t="b">
         <v>0</v>
       </c>
       <c r="O17" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2048</v>
+        <v>2051</v>
       </c>
       <c r="B18" t="s">
         <v>2034</v>
       </c>
       <c r="C18" t="n">
-        <v>1.66008471163053</v>
+        <v>1.70533676638263</v>
       </c>
       <c r="D18" t="n">
-        <v>1.18700391903699</v>
+        <v>0.816529733149712</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0350543875908492</v>
+        <v>0.00442569607457395</v>
       </c>
       <c r="F18" t="n">
-        <v>0.626700486918879</v>
+        <v>0.960149675132128</v>
       </c>
       <c r="G18" t="n">
-        <v>55</v>
+        <v>160</v>
       </c>
       <c r="H18" t="n">
-        <v>54</v>
+        <v>159</v>
       </c>
       <c r="I18" t="n">
-        <v>55</v>
+        <v>160</v>
       </c>
       <c r="J18" t="n">
-        <v>1.27046991826598</v>
+        <v>1.493749171112</v>
       </c>
       <c r="K18" t="n">
-        <v>0.382843261629623</v>
+        <v>0.0730069508591943</v>
       </c>
       <c r="L18" t="n">
-        <v>1.66008471163053</v>
+        <v>1.70533676638263</v>
       </c>
       <c r="M18" t="n">
-        <v>1.18700391903699</v>
+        <v>0.816529733149712</v>
       </c>
       <c r="N18" t="b">
         <v>0</v>
       </c>
       <c r="O18" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2049</v>
+        <v>2052</v>
       </c>
       <c r="B19" t="s">
         <v>2034</v>
       </c>
       <c r="C19" t="n">
-        <v>1.73927995059662</v>
+        <v>1.66717246170953</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.813098905337296</v>
+        <v>1.26613169537602</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0417432010170257</v>
+        <v>0.0434640611817217</v>
       </c>
       <c r="F19" t="n">
-        <v>0.93386330867079</v>
+        <v>0.551043260251077</v>
       </c>
       <c r="G19" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="H19" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="I19" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="J19" t="n">
-        <v>1.44422832824758</v>
+        <v>1.24197978950155</v>
       </c>
       <c r="K19" t="n">
-        <v>0.236574279605685</v>
+        <v>0.420793058230421</v>
       </c>
       <c r="L19" t="n">
-        <v>1.73927995059662</v>
+        <v>1.66717246170953</v>
       </c>
       <c r="M19" t="n">
-        <v>-0.813098905337296</v>
+        <v>1.26613169537602</v>
       </c>
       <c r="N19" t="b">
         <v>0</v>
       </c>
       <c r="O19" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>2050</v>
+        <v>2053</v>
       </c>
       <c r="B20" t="s">
         <v>2034</v>
       </c>
       <c r="C20" t="n">
-        <v>1.66717246170953</v>
+        <v>1.43691338176815</v>
       </c>
       <c r="D20" t="n">
-        <v>1.26613169537602</v>
+        <v>1.03333748536785</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0434640611817217</v>
+        <v>0.111414897755906</v>
       </c>
       <c r="F20" t="n">
-        <v>0.551043260251077</v>
+        <v>0.781415912832751</v>
       </c>
       <c r="G20" t="n">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="H20" t="n">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="I20" t="n">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="J20" t="n">
-        <v>1.24197978950155</v>
+        <v>1.09424738845492</v>
       </c>
       <c r="K20" t="n">
-        <v>0.420793058230421</v>
+        <v>0.564927705100365</v>
       </c>
       <c r="L20" t="n">
-        <v>1.66717246170953</v>
+        <v>1.43691338176815</v>
       </c>
       <c r="M20" t="n">
-        <v>1.26613169537602</v>
+        <v>1.03333748536785</v>
       </c>
       <c r="N20" t="b">
         <v>0</v>
       </c>
       <c r="O20" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>2051</v>
+        <v>2054</v>
       </c>
       <c r="B21" t="s">
         <v>2034</v>
       </c>
       <c r="C21" t="n">
-        <v>1.35582515562311</v>
+        <v>-0.908882442121888</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.882405625012737</v>
+        <v>-0.8211007373949</v>
       </c>
       <c r="E21" t="n">
-        <v>0.211816468982289</v>
+        <v>0.827798833558525</v>
       </c>
       <c r="F21" t="n">
-        <v>0.921121127858664</v>
+        <v>0.939529092198411</v>
       </c>
       <c r="G21" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H21" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I21" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J21" t="n">
-        <v>1.44666817087964</v>
+        <v>-0.864831842774651</v>
       </c>
       <c r="K21" t="n">
-        <v>0.209468580200288</v>
+        <v>0.874972839235664</v>
       </c>
       <c r="L21" t="n">
-        <v>1.35582515562311</v>
+        <v>-0.908882442121888</v>
       </c>
       <c r="M21" t="n">
-        <v>-0.882405625012737</v>
+        <v>-0.8211007373949</v>
       </c>
       <c r="N21" t="b">
         <v>0</v>
       </c>
       <c r="O21" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>2052</v>
+        <v>2055</v>
       </c>
       <c r="B22" t="s">
         <v>2034</v>
       </c>
       <c r="C22" t="n">
-        <v>1.65381155921971</v>
+        <v>1.66008471163053</v>
       </c>
       <c r="D22" t="n">
-        <v>-1.41637962553889</v>
+        <v>1.18700391903699</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0598891942337842</v>
+        <v>0.0350543875908492</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4479677747983</v>
+        <v>0.626700486918879</v>
       </c>
       <c r="G22" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="H22" t="n">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="I22" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="J22" t="n">
-        <v>1.88161559233992</v>
+        <v>1.27046991826598</v>
       </c>
       <c r="K22" t="n">
-        <v>0.0174534983302519</v>
+        <v>0.382843261629623</v>
       </c>
       <c r="L22" t="n">
-        <v>1.65381155921971</v>
+        <v>1.66008471163053</v>
       </c>
       <c r="M22" t="n">
-        <v>-1.41637962553889</v>
+        <v>1.18700391903699</v>
       </c>
       <c r="N22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O22" t="s">
-        <v>33</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>2053</v>
+        <v>2056</v>
       </c>
       <c r="B23" t="s">
         <v>2034</v>
       </c>
       <c r="C23" t="n">
-        <v>0.778887100366341</v>
+        <v>1.81303144165592</v>
       </c>
       <c r="D23" t="n">
-        <v>-1.02035245356723</v>
+        <v>1.93763983498075</v>
       </c>
       <c r="E23" t="n">
-        <v>0.946882388254389</v>
+        <v>0.0275455771583975</v>
       </c>
       <c r="F23" t="n">
-        <v>0.790937182749941</v>
+        <v>0.0180933176598545</v>
       </c>
       <c r="G23" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H23" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="I23" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="J23" t="n">
-        <v>1.14808621787384</v>
+        <v>-0.764179060682097</v>
       </c>
       <c r="K23" t="n">
-        <v>0.534198335931694</v>
+        <v>0.949223297337906</v>
       </c>
       <c r="L23" t="n">
-        <v>0.778887100366341</v>
+        <v>1.81303144165592</v>
       </c>
       <c r="M23" t="n">
-        <v>-1.02035245356723</v>
+        <v>1.93763983498075</v>
       </c>
       <c r="N23" t="b">
         <v>0</v>
       </c>
       <c r="O23" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>2054</v>
+        <v>2057</v>
       </c>
       <c r="B24" t="s">
         <v>2034</v>
       </c>
       <c r="C24" t="n">
-        <v>-1.01520257747063</v>
+        <v>0.858303022138855</v>
       </c>
       <c r="D24" t="n">
-        <v>1.19424185389282</v>
+        <v>-1.01846674819238</v>
       </c>
       <c r="E24" t="n">
-        <v>0.676421561638628</v>
+        <v>0.883827565913183</v>
       </c>
       <c r="F24" t="n">
-        <v>0.626700486918879</v>
+        <v>0.788383465234876</v>
       </c>
       <c r="G24" t="n">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="H24" t="n">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="I24" t="n">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="J24" t="n">
-        <v>-1.2156753146664</v>
+        <v>1.05517882825778</v>
       </c>
       <c r="K24" t="n">
-        <v>0.441817448772222</v>
+        <v>0.633959004056398</v>
       </c>
       <c r="L24" t="n">
-        <v>-1.01520257747063</v>
+        <v>0.858303022138855</v>
       </c>
       <c r="M24" t="n">
-        <v>1.19424185389282</v>
+        <v>-1.01846674819238</v>
       </c>
       <c r="N24" t="b">
         <v>0</v>
       </c>
       <c r="O24" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>2055</v>
+        <v>2058</v>
       </c>
       <c r="B25" t="s">
         <v>2034</v>
       </c>
       <c r="C25" t="n">
-        <v>1.44828403462988</v>
+        <v>-0.635856932767571</v>
       </c>
       <c r="D25" t="n">
-        <v>1.32822540349866</v>
+        <v>0.705788091270327</v>
       </c>
       <c r="E25" t="n">
-        <v>0.188568291897933</v>
+        <v>0.999054093338983</v>
       </c>
       <c r="F25" t="n">
-        <v>0.544583416703077</v>
+        <v>0.98065212751265</v>
       </c>
       <c r="G25" t="n">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="H25" t="n">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="I25" t="n">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="J25" t="n">
-        <v>-0.971477774753253</v>
+        <v>0.508125281342036</v>
       </c>
       <c r="K25" t="n">
-        <v>0.719625587265655</v>
+        <v>0.999391480730223</v>
       </c>
       <c r="L25" t="n">
-        <v>1.44828403462988</v>
+        <v>-0.635856932767571</v>
       </c>
       <c r="M25" t="n">
-        <v>1.32822540349866</v>
+        <v>0.705788091270327</v>
       </c>
       <c r="N25" t="b">
         <v>0</v>
       </c>
       <c r="O25" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>2056</v>
+        <v>2059</v>
       </c>
       <c r="B26" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.952503237797728</v>
+        <v>-1.86946782709568</v>
       </c>
       <c r="D26" t="n">
-        <v>0.687548992153339</v>
+        <v>0.719963677893052</v>
       </c>
       <c r="E26" t="n">
-        <v>0.761647518500162</v>
+        <v>0.00203304443414014</v>
       </c>
       <c r="F26" t="n">
-        <v>0.96110820624015</v>
+        <v>0.983333938876475</v>
       </c>
       <c r="G26" t="n">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="H26" t="n">
-        <v>19</v>
+        <v>96</v>
       </c>
       <c r="I26" t="n">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="J26" t="n">
-        <v>0.659655088775691</v>
+        <v>-1.657593732751</v>
       </c>
       <c r="K26" t="n">
-        <v>0.965520270340095</v>
+        <v>0.0172251263037516</v>
       </c>
       <c r="L26" t="n">
-        <v>-0.952503237797728</v>
+        <v>-1.86946782709568</v>
       </c>
       <c r="M26" t="n">
-        <v>0.687548992153339</v>
+        <v>0.719963677893052</v>
       </c>
       <c r="N26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O26" t="s">
-        <v>2036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>2057</v>
+        <v>2060</v>
       </c>
       <c r="B27" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C27" t="n">
-        <v>1.02438520348949</v>
+        <v>1.54512701694067</v>
       </c>
       <c r="D27" t="n">
-        <v>1.269710113962</v>
+        <v>1.11473681474339</v>
       </c>
       <c r="E27" t="n">
-        <v>0.661729418167425</v>
+        <v>0.12597055038879</v>
       </c>
       <c r="F27" t="n">
-        <v>0.600030808751421</v>
+        <v>0.723586415859765</v>
       </c>
       <c r="G27" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H27" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I27" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J27" t="n">
-        <v>0.927750307494303</v>
+        <v>0.954832397785224</v>
       </c>
       <c r="K27" t="n">
-        <v>0.767497746224927</v>
+        <v>0.747559323874384</v>
       </c>
       <c r="L27" t="n">
-        <v>1.02438520348949</v>
+        <v>1.54512701694067</v>
       </c>
       <c r="M27" t="n">
-        <v>1.269710113962</v>
+        <v>1.11473681474339</v>
       </c>
       <c r="N27" t="b">
         <v>0</v>
       </c>
       <c r="O27" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>2058</v>
+        <v>2061</v>
       </c>
       <c r="B28" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C28" t="n">
-        <v>-1.26575924723775</v>
+        <v>0.792618515703646</v>
       </c>
       <c r="D28" t="n">
-        <v>-1.11282892008527</v>
+        <v>0.717357540753296</v>
       </c>
       <c r="E28" t="n">
-        <v>0.305264847801037</v>
+        <v>0.919076088475296</v>
       </c>
       <c r="F28" t="n">
-        <v>0.70004508641563</v>
+        <v>0.953054194744691</v>
       </c>
       <c r="G28" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="H28" t="n">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="I28" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.704426086591038</v>
+        <v>0.649714353786492</v>
       </c>
       <c r="K28" t="n">
-        <v>0.969625345538602</v>
+        <v>0.96809157131057</v>
       </c>
       <c r="L28" t="n">
-        <v>-1.26575924723775</v>
+        <v>0.792618515703646</v>
       </c>
       <c r="M28" t="n">
-        <v>-1.11282892008527</v>
+        <v>0.717357540753296</v>
       </c>
       <c r="N28" t="b">
         <v>0</v>
       </c>
       <c r="O28" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>2059</v>
+        <v>2062</v>
       </c>
       <c r="B29" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C29" t="n">
-        <v>1.08224870181928</v>
+        <v>1.60378924675945</v>
       </c>
       <c r="D29" t="n">
-        <v>1.09639280233169</v>
+        <v>1.24069652141839</v>
       </c>
       <c r="E29" t="n">
-        <v>0.56628562092442</v>
+        <v>0.0713492013344388</v>
       </c>
       <c r="F29" t="n">
-        <v>0.733451075800617</v>
+        <v>0.602729344638531</v>
       </c>
       <c r="G29" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="H29" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="I29" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="J29" t="n">
-        <v>-0.839141635339801</v>
+        <v>0.922079154189676</v>
       </c>
       <c r="K29" t="n">
-        <v>0.901552379611377</v>
+        <v>0.800168516083537</v>
       </c>
       <c r="L29" t="n">
-        <v>1.08224870181928</v>
+        <v>1.60378924675945</v>
       </c>
       <c r="M29" t="n">
-        <v>1.09639280233169</v>
+        <v>1.24069652141839</v>
       </c>
       <c r="N29" t="b">
         <v>0</v>
       </c>
       <c r="O29" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>2060</v>
+        <v>2063</v>
       </c>
       <c r="B30" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C30" t="n">
-        <v>1.01688459917931</v>
+        <v>0.834505184754276</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.70477020001314</v>
+        <v>-0.746728001526106</v>
       </c>
       <c r="E30" t="n">
-        <v>0.683226247706747</v>
+        <v>0.890980925653246</v>
       </c>
       <c r="F30" t="n">
-        <v>0.97728842555668</v>
+        <v>0.940163423488326</v>
       </c>
       <c r="G30" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="H30" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="I30" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="J30" t="n">
-        <v>1.19954274745593</v>
+        <v>0.830417037113497</v>
       </c>
       <c r="K30" t="n">
-        <v>0.478461848697783</v>
+        <v>0.882837656017727</v>
       </c>
       <c r="L30" t="n">
-        <v>1.01688459917931</v>
+        <v>0.834505184754276</v>
       </c>
       <c r="M30" t="n">
-        <v>-0.70477020001314</v>
+        <v>-0.746728001526106</v>
       </c>
       <c r="N30" t="b">
         <v>0</v>
       </c>
       <c r="O30" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>2061</v>
+        <v>2064</v>
       </c>
       <c r="B31" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C31" t="n">
-        <v>1.43691338176815</v>
+        <v>-1.05224047280463</v>
       </c>
       <c r="D31" t="n">
-        <v>1.03333748536785</v>
+        <v>1.12308161918011</v>
       </c>
       <c r="E31" t="n">
-        <v>0.111414897755906</v>
+        <v>0.631970556862873</v>
       </c>
       <c r="F31" t="n">
-        <v>0.781415912832751</v>
+        <v>0.725703542605597</v>
       </c>
       <c r="G31" t="n">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="H31" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="I31" t="n">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="J31" t="n">
-        <v>1.09424738845492</v>
+        <v>-1.22411372522955</v>
       </c>
       <c r="K31" t="n">
-        <v>0.564927705100365</v>
+        <v>0.491191469424219</v>
       </c>
       <c r="L31" t="n">
-        <v>1.43691338176815</v>
+        <v>-1.05224047280463</v>
       </c>
       <c r="M31" t="n">
-        <v>1.03333748536785</v>
+        <v>1.12308161918011</v>
       </c>
       <c r="N31" t="b">
         <v>0</v>
       </c>
       <c r="O31" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>2062</v>
+        <v>2065</v>
       </c>
       <c r="B32" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C32" t="n">
-        <v>-0.908882442121888</v>
+        <v>0.856572036185239</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.8211007373949</v>
+        <v>-1.38308078632259</v>
       </c>
       <c r="E32" t="n">
-        <v>0.827798833558525</v>
+        <v>0.85653308816194</v>
       </c>
       <c r="F32" t="n">
-        <v>0.939529092198411</v>
+        <v>0.518418916721409</v>
       </c>
       <c r="G32" t="n">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="H32" t="n">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="I32" t="n">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="J32" t="n">
-        <v>-0.864831842774651</v>
+        <v>1.31375413322114</v>
       </c>
       <c r="K32" t="n">
-        <v>0.874972839235664</v>
+        <v>0.412099489900498</v>
       </c>
       <c r="L32" t="n">
-        <v>-0.908882442121888</v>
+        <v>0.856572036185239</v>
       </c>
       <c r="M32" t="n">
-        <v>-0.8211007373949</v>
+        <v>-1.38308078632259</v>
       </c>
       <c r="N32" t="b">
         <v>0</v>
       </c>
       <c r="O32" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>2063</v>
+        <v>2066</v>
       </c>
       <c r="B33" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C33" t="n">
-        <v>0.858303022138855</v>
+        <v>0.642885442921009</v>
       </c>
       <c r="D33" t="n">
-        <v>-1.01846674819238</v>
+        <v>1.01132503146611</v>
       </c>
       <c r="E33" t="n">
-        <v>0.883827565913183</v>
+        <v>0.995172080915972</v>
       </c>
       <c r="F33" t="n">
-        <v>0.788383465234876</v>
+        <v>0.805605329657707</v>
       </c>
       <c r="G33" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="H33" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="I33" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="J33" t="n">
-        <v>1.05517882825778</v>
+        <v>0.798040194849093</v>
       </c>
       <c r="K33" t="n">
-        <v>0.633959004056398</v>
+        <v>0.921093283753386</v>
       </c>
       <c r="L33" t="n">
-        <v>0.858303022138855</v>
+        <v>0.642885442921009</v>
       </c>
       <c r="M33" t="n">
-        <v>-1.01846674819238</v>
+        <v>1.01132503146611</v>
       </c>
       <c r="N33" t="b">
         <v>0</v>
       </c>
       <c r="O33" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>2064</v>
+        <v>2067</v>
       </c>
       <c r="B34" t="s">
-        <v>2034</v>
+        <v>1930</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.635856932767571</v>
+        <v>0.729483137227436</v>
       </c>
       <c r="D34" t="n">
-        <v>0.705788091270327</v>
+        <v>1.67379586129908</v>
       </c>
       <c r="E34" t="n">
-        <v>0.999054093338983</v>
+        <v>0.967718113618937</v>
       </c>
       <c r="F34" t="n">
-        <v>0.98065212751265</v>
+        <v>0.166278960600023</v>
       </c>
       <c r="G34" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="H34" t="n">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="I34" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="J34" t="n">
-        <v>0.508125281342036</v>
+        <v>-1.36125939000036</v>
       </c>
       <c r="K34" t="n">
-        <v>0.999391480730223</v>
+        <v>0.337096561657965</v>
       </c>
       <c r="L34" t="n">
-        <v>-0.635856932767571</v>
+        <v>0.729483137227436</v>
       </c>
       <c r="M34" t="n">
-        <v>0.705788091270327</v>
+        <v>1.67379586129908</v>
       </c>
       <c r="N34" t="b">
         <v>0</v>
       </c>
       <c r="O34" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>2065</v>
+        <v>2068</v>
       </c>
       <c r="B35" t="s">
         <v>1930</v>
       </c>
       <c r="C35" t="n">
-        <v>1.54512701694067</v>
+        <v>1.8999377038983</v>
       </c>
       <c r="D35" t="n">
-        <v>1.11473681474339</v>
+        <v>1.87146635592682</v>
       </c>
       <c r="E35" t="n">
-        <v>0.12597055038879</v>
+        <v>0.00888284792363617</v>
       </c>
       <c r="F35" t="n">
-        <v>0.723586415859765</v>
+        <v>0.0446591031563833</v>
       </c>
       <c r="G35" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H35" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I35" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J35" t="n">
-        <v>0.954832397785224</v>
+        <v>1.04770669503782</v>
       </c>
       <c r="K35" t="n">
-        <v>0.747559323874384</v>
+        <v>0.641277702659038</v>
       </c>
       <c r="L35" t="n">
-        <v>1.54512701694067</v>
+        <v>1.8999377038983</v>
       </c>
       <c r="M35" t="n">
-        <v>1.11473681474339</v>
+        <v>1.87146635592682</v>
       </c>
       <c r="N35" t="b">
         <v>0</v>
       </c>
       <c r="O35" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>2066</v>
+        <v>2069</v>
       </c>
       <c r="B36" t="s">
         <v>1930</v>
       </c>
       <c r="C36" t="n">
-        <v>0.792618515703646</v>
+        <v>-0.506232363785937</v>
       </c>
       <c r="D36" t="n">
-        <v>0.717357540753296</v>
+        <v>-0.659556875009062</v>
       </c>
       <c r="E36" t="n">
-        <v>0.919076088475296</v>
+        <v>0.999599358974359</v>
       </c>
       <c r="F36" t="n">
-        <v>0.953054194744691</v>
+        <v>0.983333938876475</v>
       </c>
       <c r="G36" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="H36" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="I36" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="J36" t="n">
-        <v>0.649714353786492</v>
+        <v>-0.58902413920141</v>
       </c>
       <c r="K36" t="n">
-        <v>0.96809157131057</v>
+        <v>0.989796956316857</v>
       </c>
       <c r="L36" t="n">
-        <v>0.792618515703646</v>
+        <v>-0.506232363785937</v>
       </c>
       <c r="M36" t="n">
-        <v>0.717357540753296</v>
+        <v>-0.659556875009062</v>
       </c>
       <c r="N36" t="b">
         <v>0</v>
       </c>
       <c r="O36" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>2067</v>
+        <v>2070</v>
       </c>
       <c r="B37" t="s">
         <v>1930</v>
       </c>
       <c r="C37" t="n">
-        <v>1.60378924675945</v>
+        <v>-0.565561050800147</v>
       </c>
       <c r="D37" t="n">
-        <v>1.24069652141839</v>
+        <v>1.50418060203554</v>
       </c>
       <c r="E37" t="n">
-        <v>0.0713492013344388</v>
+        <v>0.999054093338983</v>
       </c>
       <c r="F37" t="n">
-        <v>0.602729344638531</v>
+        <v>0.364010047956154</v>
       </c>
       <c r="G37" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H37" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="I37" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="J37" t="n">
-        <v>0.922079154189676</v>
+        <v>-1.39865642925211</v>
       </c>
       <c r="K37" t="n">
-        <v>0.800168516083537</v>
+        <v>0.345514309245917</v>
       </c>
       <c r="L37" t="n">
-        <v>1.60378924675945</v>
+        <v>-0.565561050800147</v>
       </c>
       <c r="M37" t="n">
-        <v>1.24069652141839</v>
+        <v>1.50418060203554</v>
       </c>
       <c r="N37" t="b">
         <v>0</v>
       </c>
       <c r="O37" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>2068</v>
+        <v>2071</v>
       </c>
       <c r="B38" t="s">
         <v>1930</v>
       </c>
       <c r="C38" t="n">
-        <v>0.834505184754276</v>
+        <v>0.771128607902183</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.746728001526106</v>
+        <v>1.20794006152421</v>
       </c>
       <c r="E38" t="n">
-        <v>0.890980925653246</v>
+        <v>0.947266208459145</v>
       </c>
       <c r="F38" t="n">
-        <v>0.940163423488326</v>
+        <v>0.635966741577025</v>
       </c>
       <c r="G38" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="H38" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I38" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="J38" t="n">
-        <v>0.830417037113497</v>
+        <v>-0.815595567377427</v>
       </c>
       <c r="K38" t="n">
-        <v>0.882837656017727</v>
+        <v>0.904130623390176</v>
       </c>
       <c r="L38" t="n">
-        <v>0.834505184754276</v>
+        <v>0.771128607902183</v>
       </c>
       <c r="M38" t="n">
-        <v>-0.746728001526106</v>
+        <v>1.20794006152421</v>
       </c>
       <c r="N38" t="b">
         <v>0</v>
       </c>
       <c r="O38" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>2069</v>
+        <v>1949</v>
       </c>
       <c r="B39" t="s">
         <v>1930</v>
       </c>
       <c r="C39" t="n">
-        <v>-1.05224047280463</v>
+        <v>-2.09530870215646</v>
       </c>
       <c r="D39" t="n">
-        <v>1.12308161918011</v>
+        <v>-0.88328325844714</v>
       </c>
       <c r="E39" t="n">
-        <v>0.631970556862873</v>
+        <v>0.0000737780828421685</v>
       </c>
       <c r="F39" t="n">
-        <v>0.725703542605597</v>
+        <v>0.924770700656501</v>
       </c>
       <c r="G39" t="n">
-        <v>20</v>
+        <v>86</v>
       </c>
       <c r="H39" t="n">
-        <v>20</v>
+        <v>86</v>
       </c>
       <c r="I39" t="n">
-        <v>20</v>
+        <v>86</v>
       </c>
       <c r="J39" t="n">
-        <v>-1.22411372522955</v>
+        <v>-1.71677175976851</v>
       </c>
       <c r="K39" t="n">
-        <v>0.491191469424219</v>
+        <v>0.0174534983302519</v>
       </c>
       <c r="L39" t="n">
-        <v>-1.05224047280463</v>
+        <v>-2.09530870215646</v>
       </c>
       <c r="M39" t="n">
-        <v>1.12308161918011</v>
+        <v>-0.88328325844714</v>
       </c>
       <c r="N39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O39" t="s">
-        <v>2036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>2070</v>
+        <v>2072</v>
       </c>
       <c r="B40" t="s">
         <v>1930</v>
       </c>
       <c r="C40" t="n">
-        <v>0.856572036185239</v>
+        <v>2.19134060699225</v>
       </c>
       <c r="D40" t="n">
-        <v>-1.38308078632259</v>
+        <v>1.0754110538426</v>
       </c>
       <c r="E40" t="n">
-        <v>0.85653308816194</v>
+        <v>0.000645051063205934</v>
       </c>
       <c r="F40" t="n">
-        <v>0.518418916721409</v>
+        <v>0.746714126712962</v>
       </c>
       <c r="G40" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="H40" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="I40" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="J40" t="n">
-        <v>1.31375413322114</v>
+        <v>1.95896018601054</v>
       </c>
       <c r="K40" t="n">
-        <v>0.412099489900498</v>
+        <v>0.0145465812893292</v>
       </c>
       <c r="L40" t="n">
-        <v>0.856572036185239</v>
+        <v>2.19134060699225</v>
       </c>
       <c r="M40" t="n">
-        <v>-1.38308078632259</v>
+        <v>1.0754110538426</v>
       </c>
       <c r="N40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O40" t="s">
-        <v>2036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>2071</v>
+        <v>2073</v>
       </c>
       <c r="B41" t="s">
         <v>1930</v>
       </c>
       <c r="C41" t="n">
-        <v>0.642885442921009</v>
+        <v>-1.76363136225828</v>
       </c>
       <c r="D41" t="n">
-        <v>1.01132503146611</v>
+        <v>0.873534564896149</v>
       </c>
       <c r="E41" t="n">
-        <v>0.995172080915972</v>
+        <v>0.0114942849232801</v>
       </c>
       <c r="F41" t="n">
-        <v>0.805605329657707</v>
+        <v>0.921121127858664</v>
       </c>
       <c r="G41" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="H41" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="I41" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="J41" t="n">
-        <v>0.798040194849093</v>
+        <v>-1.64855500834541</v>
       </c>
       <c r="K41" t="n">
-        <v>0.921093283753386</v>
+        <v>0.0736698325163399</v>
       </c>
       <c r="L41" t="n">
-        <v>0.642885442921009</v>
+        <v>-1.76363136225828</v>
       </c>
       <c r="M41" t="n">
-        <v>1.01132503146611</v>
+        <v>0.873534564896149</v>
       </c>
       <c r="N41" t="b">
         <v>0</v>
       </c>
       <c r="O41" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>2072</v>
+        <v>1975</v>
       </c>
       <c r="B42" t="s">
         <v>1930</v>
       </c>
       <c r="C42" t="n">
-        <v>0.729483137227436</v>
+        <v>-0.974037439552858</v>
       </c>
       <c r="D42" t="n">
-        <v>1.67379586129908</v>
+        <v>2.75091489958207</v>
       </c>
       <c r="E42" t="n">
-        <v>0.967718113618937</v>
+        <v>0.732097622100758</v>
       </c>
       <c r="F42" t="n">
-        <v>0.166278960600023</v>
+        <v>0.0000000000419946215141542</v>
       </c>
       <c r="G42" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="H42" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="I42" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="J42" t="n">
-        <v>-1.36125939000036</v>
+        <v>-2.73153008004191</v>
       </c>
       <c r="K42" t="n">
-        <v>0.337096561657965</v>
+        <v>0.00000000964910699071031</v>
       </c>
       <c r="L42" t="n">
-        <v>0.729483137227436</v>
+        <v>-0.974037439552858</v>
       </c>
       <c r="M42" t="n">
-        <v>1.67379586129908</v>
+        <v>2.75091489958207</v>
       </c>
       <c r="N42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O42" t="s">
-        <v>2036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>2073</v>
+        <v>2074</v>
       </c>
       <c r="B43" t="s">
         <v>1930</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.506232363785937</v>
+        <v>0.911605384205958</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.659556875009062</v>
+        <v>0.903412694647803</v>
       </c>
       <c r="E43" t="n">
-        <v>0.999599358974359</v>
+        <v>0.813903521067077</v>
       </c>
       <c r="F43" t="n">
-        <v>0.983333938876475</v>
+        <v>0.897636591817711</v>
       </c>
       <c r="G43" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="H43" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="I43" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J43" t="n">
-        <v>-0.58902413920141</v>
+        <v>-1.10256434229325</v>
       </c>
       <c r="K43" t="n">
-        <v>0.989796956316857</v>
+        <v>0.58250920679488</v>
       </c>
       <c r="L43" t="n">
-        <v>-0.506232363785937</v>
+        <v>0.911605384205958</v>
       </c>
       <c r="M43" t="n">
-        <v>-0.659556875009062</v>
+        <v>0.903412694647803</v>
       </c>
       <c r="N43" t="b">
         <v>0</v>
       </c>
       <c r="O43" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>2074</v>
+        <v>2075</v>
       </c>
       <c r="B44" t="s">
         <v>1930</v>
       </c>
       <c r="C44" t="n">
-        <v>-0.565561050800147</v>
+        <v>0.641698585640167</v>
       </c>
       <c r="D44" t="n">
-        <v>1.50418060203554</v>
+        <v>1.24775221906794</v>
       </c>
       <c r="E44" t="n">
-        <v>0.999054093338983</v>
+        <v>0.991557670194802</v>
       </c>
       <c r="F44" t="n">
-        <v>0.364010047956154</v>
+        <v>0.620719099530415</v>
       </c>
       <c r="G44" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H44" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I44" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="J44" t="n">
-        <v>-1.39865642925211</v>
+        <v>-1.1517190824162</v>
       </c>
       <c r="K44" t="n">
-        <v>0.345514309245917</v>
+        <v>0.547045412756838</v>
       </c>
       <c r="L44" t="n">
-        <v>-0.565561050800147</v>
+        <v>0.641698585640167</v>
       </c>
       <c r="M44" t="n">
-        <v>1.50418060203554</v>
+        <v>1.24775221906794</v>
       </c>
       <c r="N44" t="b">
         <v>0</v>
       </c>
       <c r="O44" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>2075</v>
+        <v>2076</v>
       </c>
       <c r="B45" t="s">
         <v>1930</v>
       </c>
       <c r="C45" t="n">
-        <v>0.771128607902183</v>
+        <v>0.991097942767018</v>
       </c>
       <c r="D45" t="n">
-        <v>1.20794006152421</v>
+        <v>1.66017957238675</v>
       </c>
       <c r="E45" t="n">
-        <v>0.947266208459145</v>
+        <v>0.708571900644588</v>
       </c>
       <c r="F45" t="n">
-        <v>0.635966741577025</v>
+        <v>0.179831593773824</v>
       </c>
       <c r="G45" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="H45" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="I45" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="J45" t="n">
-        <v>-0.815595567377427</v>
+        <v>-1.15973437129099</v>
       </c>
       <c r="K45" t="n">
-        <v>0.904130623390176</v>
+        <v>0.549038366581078</v>
       </c>
       <c r="L45" t="n">
-        <v>0.771128607902183</v>
+        <v>0.991097942767018</v>
       </c>
       <c r="M45" t="n">
-        <v>1.20794006152421</v>
+        <v>1.66017957238675</v>
       </c>
       <c r="N45" t="b">
         <v>0</v>
       </c>
       <c r="O45" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>1975</v>
+        <v>2077</v>
       </c>
       <c r="B46" t="s">
         <v>1930</v>
       </c>
       <c r="C46" t="n">
-        <v>-0.974037439552858</v>
+        <v>1.97676024961818</v>
       </c>
       <c r="D46" t="n">
-        <v>2.75091489958207</v>
+        <v>-0.653603238796788</v>
       </c>
       <c r="E46" t="n">
-        <v>0.732097622100758</v>
+        <v>0.00482063296372364</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0000000000419946215141542</v>
+        <v>0.983333938876475</v>
       </c>
       <c r="G46" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="H46" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="I46" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="J46" t="n">
-        <v>-2.73153008004191</v>
+        <v>1.83429777592081</v>
       </c>
       <c r="K46" t="n">
-        <v>0.00000000964910699071031</v>
+        <v>0.0272926051995232</v>
       </c>
       <c r="L46" t="n">
-        <v>-0.974037439552858</v>
+        <v>1.97676024961818</v>
       </c>
       <c r="M46" t="n">
-        <v>2.75091489958207</v>
+        <v>-0.653603238796788</v>
       </c>
       <c r="N46" t="b">
         <v>1</v>
@@ -62269,190 +62269,190 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>2076</v>
+        <v>2078</v>
       </c>
       <c r="B47" t="s">
         <v>1930</v>
       </c>
       <c r="C47" t="n">
-        <v>0.911605384205958</v>
+        <v>0.900022709170423</v>
       </c>
       <c r="D47" t="n">
-        <v>0.903412694647803</v>
+        <v>1.56729902261791</v>
       </c>
       <c r="E47" t="n">
-        <v>0.813903521067077</v>
+        <v>0.858077998568708</v>
       </c>
       <c r="F47" t="n">
-        <v>0.897636591817711</v>
+        <v>0.133020280754935</v>
       </c>
       <c r="G47" t="n">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="H47" t="n">
-        <v>45</v>
+        <v>83</v>
       </c>
       <c r="I47" t="n">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="J47" t="n">
-        <v>-1.10256434229325</v>
+        <v>-1.4488937243172</v>
       </c>
       <c r="K47" t="n">
-        <v>0.58250920679488</v>
+        <v>0.14846381660751</v>
       </c>
       <c r="L47" t="n">
-        <v>0.911605384205958</v>
+        <v>0.900022709170423</v>
       </c>
       <c r="M47" t="n">
-        <v>0.903412694647803</v>
+        <v>1.56729902261791</v>
       </c>
       <c r="N47" t="b">
         <v>0</v>
       </c>
       <c r="O47" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>2077</v>
+        <v>1928</v>
       </c>
       <c r="B48" t="s">
         <v>1930</v>
       </c>
       <c r="C48" t="n">
-        <v>0.641698585640167</v>
+        <v>2.17641704034345</v>
       </c>
       <c r="D48" t="n">
-        <v>1.24775221906794</v>
+        <v>1.72909466449593</v>
       </c>
       <c r="E48" t="n">
-        <v>0.991557670194802</v>
+        <v>0.00000430594823680413</v>
       </c>
       <c r="F48" t="n">
-        <v>0.620719099530415</v>
+        <v>0.024475642139805</v>
       </c>
       <c r="G48" t="n">
-        <v>23</v>
+        <v>119</v>
       </c>
       <c r="H48" t="n">
-        <v>23</v>
+        <v>118</v>
       </c>
       <c r="I48" t="n">
-        <v>23</v>
+        <v>119</v>
       </c>
       <c r="J48" t="n">
-        <v>-1.1517190824162</v>
+        <v>1.31472586306208</v>
       </c>
       <c r="K48" t="n">
-        <v>0.547045412756838</v>
+        <v>0.253696621162633</v>
       </c>
       <c r="L48" t="n">
-        <v>0.641698585640167</v>
+        <v>2.17641704034345</v>
       </c>
       <c r="M48" t="n">
-        <v>1.24775221906794</v>
+        <v>1.72909466449593</v>
       </c>
       <c r="N48" t="b">
         <v>0</v>
       </c>
       <c r="O48" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>2078</v>
+        <v>2079</v>
       </c>
       <c r="B49" t="s">
         <v>1930</v>
       </c>
       <c r="C49" t="n">
-        <v>0.991097942767018</v>
+        <v>0.925995839314815</v>
       </c>
       <c r="D49" t="n">
-        <v>1.66017957238675</v>
+        <v>-0.818675947262084</v>
       </c>
       <c r="E49" t="n">
-        <v>0.708571900644588</v>
+        <v>0.819885481058537</v>
       </c>
       <c r="F49" t="n">
-        <v>0.179831593773824</v>
+        <v>0.953054194744691</v>
       </c>
       <c r="G49" t="n">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="H49" t="n">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="I49" t="n">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="J49" t="n">
-        <v>-1.15973437129099</v>
+        <v>1.06145725062268</v>
       </c>
       <c r="K49" t="n">
-        <v>0.549038366581078</v>
+        <v>0.616994811663881</v>
       </c>
       <c r="L49" t="n">
-        <v>0.991097942767018</v>
+        <v>0.925995839314815</v>
       </c>
       <c r="M49" t="n">
-        <v>1.66017957238675</v>
+        <v>-0.818675947262084</v>
       </c>
       <c r="N49" t="b">
         <v>0</v>
       </c>
       <c r="O49" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>2079</v>
+        <v>1939</v>
       </c>
       <c r="B50" t="s">
         <v>1930</v>
       </c>
       <c r="C50" t="n">
-        <v>0.900022709170423</v>
+        <v>-2.65625893338279</v>
       </c>
       <c r="D50" t="n">
-        <v>1.56729902261791</v>
+        <v>-1.38159490915102</v>
       </c>
       <c r="E50" t="n">
-        <v>0.858077998568708</v>
+        <v>0.000000000000947150908861262</v>
       </c>
       <c r="F50" t="n">
-        <v>0.133020280754935</v>
+        <v>0.207765658228716</v>
       </c>
       <c r="G50" t="n">
-        <v>83</v>
+        <v>152</v>
       </c>
       <c r="H50" t="n">
-        <v>83</v>
+        <v>152</v>
       </c>
       <c r="I50" t="n">
-        <v>83</v>
+        <v>152</v>
       </c>
       <c r="J50" t="n">
-        <v>-1.4488937243172</v>
+        <v>-1.79082687996285</v>
       </c>
       <c r="K50" t="n">
-        <v>0.14846381660751</v>
+        <v>0.00189151757306219</v>
       </c>
       <c r="L50" t="n">
-        <v>0.900022709170423</v>
+        <v>-2.65625893338279</v>
       </c>
       <c r="M50" t="n">
-        <v>1.56729902261791</v>
+        <v>-1.38159490915102</v>
       </c>
       <c r="N50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O50" t="s">
-        <v>2036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="51">
@@ -62463,43 +62463,43 @@
         <v>1930</v>
       </c>
       <c r="C51" t="n">
-        <v>0.925995839314815</v>
+        <v>-1.00135782040305</v>
       </c>
       <c r="D51" t="n">
-        <v>-0.818675947262084</v>
+        <v>1.03430019592493</v>
       </c>
       <c r="E51" t="n">
-        <v>0.819885481058537</v>
+        <v>0.698148314686196</v>
       </c>
       <c r="F51" t="n">
-        <v>0.953054194744691</v>
+        <v>0.791179908419798</v>
       </c>
       <c r="G51" t="n">
-        <v>94</v>
+        <v>23</v>
       </c>
       <c r="H51" t="n">
-        <v>94</v>
+        <v>23</v>
       </c>
       <c r="I51" t="n">
-        <v>94</v>
+        <v>23</v>
       </c>
       <c r="J51" t="n">
-        <v>1.06145725062268</v>
+        <v>-1.06513561246436</v>
       </c>
       <c r="K51" t="n">
-        <v>0.616994811663881</v>
+        <v>0.633959004056398</v>
       </c>
       <c r="L51" t="n">
-        <v>0.925995839314815</v>
+        <v>-1.00135782040305</v>
       </c>
       <c r="M51" t="n">
-        <v>-0.818675947262084</v>
+        <v>1.03430019592493</v>
       </c>
       <c r="N51" t="b">
         <v>0</v>
       </c>
       <c r="O51" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="52">
@@ -62510,43 +62510,43 @@
         <v>1930</v>
       </c>
       <c r="C52" t="n">
-        <v>-1.00135782040305</v>
+        <v>-1.30653152194421</v>
       </c>
       <c r="D52" t="n">
-        <v>1.03430019592493</v>
+        <v>-0.860501052531911</v>
       </c>
       <c r="E52" t="n">
-        <v>0.698148314686196</v>
+        <v>0.281566375961631</v>
       </c>
       <c r="F52" t="n">
-        <v>0.791179908419798</v>
+        <v>0.921121127858664</v>
       </c>
       <c r="G52" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="H52" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="I52" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="J52" t="n">
-        <v>-1.06513561246436</v>
+        <v>-1.04239983594238</v>
       </c>
       <c r="K52" t="n">
-        <v>0.633959004056398</v>
+        <v>0.644149771749429</v>
       </c>
       <c r="L52" t="n">
-        <v>-1.00135782040305</v>
+        <v>-1.30653152194421</v>
       </c>
       <c r="M52" t="n">
-        <v>1.03430019592493</v>
+        <v>-0.860501052531911</v>
       </c>
       <c r="N52" t="b">
         <v>0</v>
       </c>
       <c r="O52" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="53">
@@ -62557,16 +62557,16 @@
         <v>1930</v>
       </c>
       <c r="C53" t="n">
-        <v>-1.30653152194421</v>
+        <v>1.05448105961049</v>
       </c>
       <c r="D53" t="n">
-        <v>-0.860501052531911</v>
+        <v>1.05431475837936</v>
       </c>
       <c r="E53" t="n">
-        <v>0.281566375961631</v>
+        <v>0.631970556862873</v>
       </c>
       <c r="F53" t="n">
-        <v>0.921121127858664</v>
+        <v>0.759578689862603</v>
       </c>
       <c r="G53" t="n">
         <v>36</v>
@@ -62578,22 +62578,22 @@
         <v>36</v>
       </c>
       <c r="J53" t="n">
-        <v>-1.04239983594238</v>
+        <v>-0.860602806032806</v>
       </c>
       <c r="K53" t="n">
-        <v>0.644149771749429</v>
+        <v>0.869337785402643</v>
       </c>
       <c r="L53" t="n">
-        <v>-1.30653152194421</v>
+        <v>1.05448105961049</v>
       </c>
       <c r="M53" t="n">
-        <v>-0.860501052531911</v>
+        <v>1.05431475837936</v>
       </c>
       <c r="N53" t="b">
         <v>0</v>
       </c>
       <c r="O53" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="54">
@@ -62604,43 +62604,43 @@
         <v>1930</v>
       </c>
       <c r="C54" t="n">
-        <v>1.05448105961049</v>
+        <v>1.26816347230059</v>
       </c>
       <c r="D54" t="n">
-        <v>1.05431475837936</v>
+        <v>-0.973425815013731</v>
       </c>
       <c r="E54" t="n">
-        <v>0.631970556862873</v>
+        <v>0.319454172499734</v>
       </c>
       <c r="F54" t="n">
-        <v>0.759578689862603</v>
+        <v>0.830829098966833</v>
       </c>
       <c r="G54" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H54" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I54" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J54" t="n">
-        <v>-0.860602806032806</v>
+        <v>1.38610538500767</v>
       </c>
       <c r="K54" t="n">
-        <v>0.869337785402643</v>
+        <v>0.288668491893529</v>
       </c>
       <c r="L54" t="n">
-        <v>1.05448105961049</v>
+        <v>1.26816347230059</v>
       </c>
       <c r="M54" t="n">
-        <v>1.05431475837936</v>
+        <v>-0.973425815013731</v>
       </c>
       <c r="N54" t="b">
         <v>0</v>
       </c>
       <c r="O54" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="55">
@@ -62651,43 +62651,43 @@
         <v>1930</v>
       </c>
       <c r="C55" t="n">
-        <v>1.26816347230059</v>
+        <v>1.27160692750321</v>
       </c>
       <c r="D55" t="n">
-        <v>-0.973425815013731</v>
+        <v>1.7945280201667</v>
       </c>
       <c r="E55" t="n">
-        <v>0.319454172499734</v>
+        <v>0.361852498160461</v>
       </c>
       <c r="F55" t="n">
-        <v>0.830829098966833</v>
+        <v>0.121232144665727</v>
       </c>
       <c r="G55" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="H55" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="I55" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="J55" t="n">
-        <v>1.38610538500767</v>
+        <v>-1.20230798660857</v>
       </c>
       <c r="K55" t="n">
-        <v>0.288668491893529</v>
+        <v>0.503914674075887</v>
       </c>
       <c r="L55" t="n">
-        <v>1.26816347230059</v>
+        <v>1.27160692750321</v>
       </c>
       <c r="M55" t="n">
-        <v>-0.973425815013731</v>
+        <v>1.7945280201667</v>
       </c>
       <c r="N55" t="b">
         <v>0</v>
       </c>
       <c r="O55" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="56">
@@ -62698,43 +62698,43 @@
         <v>1930</v>
       </c>
       <c r="C56" t="n">
-        <v>1.27160692750321</v>
+        <v>2.0843779279202</v>
       </c>
       <c r="D56" t="n">
-        <v>1.7945280201667</v>
+        <v>-1.13354216006671</v>
       </c>
       <c r="E56" t="n">
-        <v>0.361852498160461</v>
+        <v>0.00214014985753382</v>
       </c>
       <c r="F56" t="n">
-        <v>0.121232144665727</v>
+        <v>0.691622761470133</v>
       </c>
       <c r="G56" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H56" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="I56" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="J56" t="n">
-        <v>-1.20230798660857</v>
+        <v>2.17554919441156</v>
       </c>
       <c r="K56" t="n">
-        <v>0.503914674075887</v>
+        <v>0.00157336216247884</v>
       </c>
       <c r="L56" t="n">
-        <v>1.27160692750321</v>
+        <v>2.0843779279202</v>
       </c>
       <c r="M56" t="n">
-        <v>1.7945280201667</v>
+        <v>-1.13354216006671</v>
       </c>
       <c r="N56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O56" t="s">
-        <v>2036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="57">
@@ -62781,7 +62781,7 @@
         <v>0</v>
       </c>
       <c r="O57" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="58">
@@ -62828,7 +62828,7 @@
         <v>0</v>
       </c>
       <c r="O58" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
     </row>
   </sheetData>

</xml_diff>